<commit_message>
chore(data): trait translations, voice console handling, mzh/prune scripts
- Translate more character traits to Chinese in the client label map
- VNDB voice data: prefer original (non-console) voice actors per character
- Add measure-mzh-coverage and prune-missing-trait-characters maintenance scripts
- Add matching pnpm scripts and update 游戏名.xlsx data
</commit_message>
<xml_diff>
--- a/scripts/游戏名.xlsx
+++ b/scripts/游戏名.xlsx
@@ -780,7 +780,7 @@
       </c>
       <c r="Z3" s="1" t="inlineStr">
         <is>
-          <t>秦 且歌、赵 爽、苗洋、桑 毓泽、陈 婷婷</t>
+          <t>秦 且歌、赵 爽、桑 毓泽、陈 婷婷</t>
         </is>
       </c>
       <c r="AA3" s="1" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="Z9" s="1" t="inlineStr">
         <is>
-          <t>加隈 亜衣、広瀬 裕也、山根 綺、Lynn、関根 瞳、藍本 あみ</t>
+          <t>加隈 亜衣、広瀬 裕也、山根 綺、\N、関根 瞳、藍本 あみ</t>
         </is>
       </c>
       <c r="AA9" s="1" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="Z16" s="1" t="inlineStr">
         <is>
-          <t>加隈 亜衣、秋野 花、月野 きいろ、相模 恋、小波 すず、天知 遥、石見 舞菜香、小岩井ことり、関根 明良、古賀 葵</t>
+          <t>加隈 亜衣、秋野 花、月野 きいろ、相模 恋、小波 すず</t>
         </is>
       </c>
       <c r="AA16" s="1" t="inlineStr">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="Z20" s="1" t="inlineStr">
         <is>
-          <t>明羽 杏子</t>
+          <t>明羽 杏子、都 とわ</t>
         </is>
       </c>
       <c r="AA20" s="1" t="inlineStr">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="Z21" s="1" t="inlineStr">
         <is>
-          <t>越 雪光、手塚 りょうこ、綾音 まこ、夏和小、広山 和重</t>
+          <t>越 雪光、桜川 未央、澤田 なつ、五行 なずな、手塚 りょうこ、綾音 まこ、藤神 司朗、夏和小、広山 和重</t>
         </is>
       </c>
       <c r="AA21" s="1" t="inlineStr">
@@ -3413,7 +3413,7 @@
       </c>
       <c r="Z28" s="1" t="inlineStr">
         <is>
-          <t>柳 知萧、月夜桥、森中人、海棠不言、赵 爽</t>
+          <t>柳 知萧、月夜桥、森中人、赵 爽</t>
         </is>
       </c>
       <c r="AA28" s="1" t="inlineStr">
@@ -3720,7 +3720,7 @@
       </c>
       <c r="Z31" s="1" t="inlineStr">
         <is>
-          <t>奏雨、小山 さほみ、花澤 さくら、小波 すず、梅木 ちはる、東 シヅ</t>
+          <t>奏雨、御苑生 メイ、花澤 さくら、小波 すず、梅木 ちはる、東 シヅ</t>
         </is>
       </c>
       <c r="AA31" s="1" t="inlineStr">
@@ -4186,7 +4186,7 @@
       </c>
       <c r="Z35" s="1" t="inlineStr">
         <is>
-          <t>尾狐殿、师欣、紫丞少主、阿戈伊奥、傻莓酱、Geass、Kenz、妖女、岚风蜂蜜绿茶、百劫星罗</t>
+          <t>尾狐殿、师欣、紫丞少主、阿戈伊奥、傻莓酱、\N、\N、妖女、岚风蜂蜜绿茶、百劫星罗</t>
         </is>
       </c>
       <c r="AA35" s="1" t="inlineStr">
@@ -5396,7 +5396,7 @@
       </c>
       <c r="Z46" s="1" t="inlineStr">
         <is>
-          <t>秋野 花、戸田 めぐみ、堀場 美希、紬 雪乃</t>
+          <t>秋野 花、柳 ひとみ、浜辺 実雨、紬 雪乃</t>
         </is>
       </c>
       <c r="AA46" s="1" t="inlineStr">
@@ -5608,7 +5608,7 @@
           <t>MANYO、aya Sueki、Jerome Kern</t>
         </is>
       </c>
-      <c r="Z48" t="inlineStr">
+      <c r="Z48" s="0" t="inlineStr">
         <is>
           <t>柚木 かなめ、葉村 夏緒、秋城 柚月、かわしま りの、滝沢 アツヤ、Back麗男、原田 友貴、機知 通、河村 眞人、髭内 悪太</t>
         </is>
@@ -6235,7 +6235,7 @@
       </c>
       <c r="Z54" s="1" t="inlineStr">
         <is>
-          <t>遥 そら、奏雨、杏子 御津、歩 サラ、白雪 碧、くすはら ゆい、阿澄 佳奈、加藤 英美里、水瀬 いのり、東山 奈央、結城 ほのか、伊藤 彩沙、前川 涼子、尾崎 由香</t>
+          <t>遥 そら、奏雨、杏子 御津、歩 サラ、白雪 碧、くすはら ゆい、加藤 英美里</t>
         </is>
       </c>
       <c r="AA54" s="1" t="inlineStr">
@@ -7129,7 +7129,7 @@
           <t>虻川 治、堀江 晶太</t>
         </is>
       </c>
-      <c r="Z62" t="inlineStr">
+      <c r="Z62" s="0" t="inlineStr">
         <is>
           <t>澤田 なつ、寺竹 順、沢澤 砂羽、夏和小、渚 しろな</t>
         </is>
@@ -7464,7 +7464,7 @@
       </c>
       <c r="Z65" s="1" t="inlineStr">
         <is>
-          <t>沢野 ぽぷら、わらび 茶々</t>
+          <t>花澤 さくら、そらまめ。、沢野 ぽぷら、わらび 茶々、水野 七海、柳 ひとみ、こはる 凪、飴川 紫乃、倉田 ありあ</t>
         </is>
       </c>
       <c r="AA65" s="1" t="inlineStr">
@@ -9205,7 +9205,7 @@
           <t>安瀬 聖、虻川 治</t>
         </is>
       </c>
-      <c r="Z81" t="inlineStr">
+      <c r="Z81" s="0" t="inlineStr">
         <is>
           <t>澤田 なつ、寺竹 順、沢澤 砂羽、夏和小、渚 しろな</t>
         </is>
@@ -9510,7 +9510,7 @@
       </c>
       <c r="Z84" s="1" t="inlineStr">
         <is>
-          <t>小野 涼子、小波 すず、蒼乃 むすび、飴川 紫乃</t>
+          <t>北見 六花、小波 すず、蒼乃 むすび、飴川 紫乃</t>
         </is>
       </c>
       <c r="AA84" s="1" t="inlineStr">
@@ -9813,7 +9813,7 @@
           <t>水城 新人、Team-OZ、山田 重利、Shinji、PHA、Henry Clay Work</t>
         </is>
       </c>
-      <c r="Z87" t="inlineStr">
+      <c r="Z87" s="0" t="inlineStr">
         <is>
           <t>小倉 結衣、有坂 羽由</t>
         </is>
@@ -9919,7 +9919,7 @@
       </c>
       <c r="Z88" s="1" t="inlineStr">
         <is>
-          <t>石上 静香、雨場 つかさ</t>
+          <t>大橋 歩夕、石上 静香、大地 葉、山岡 ゆり、雨場 つかさ</t>
         </is>
       </c>
       <c r="AA88" s="1" t="inlineStr">
@@ -10022,7 +10022,7 @@
           <t>電気式華憐音楽集団、電気、Gaku</t>
         </is>
       </c>
-      <c r="Z89" t="inlineStr">
+      <c r="Z89" s="0" t="inlineStr">
         <is>
           <t>藤森 ゆき奈、榛名 れん、白月 かなめ、苺山 文太郎、仙地 祐里衣</t>
         </is>
@@ -10342,7 +10342,7 @@
       </c>
       <c r="Z92" s="1" t="inlineStr">
         <is>
-          <t>清水 愛、加藤 英美里、荒浪 和沙、上坂 すみれ、戸田 めぐみ、清水 彩香、桐谷 蝶々、藤田 昌代、桑原 由気、村上 奈津実、鈴代 紗弓</t>
+          <t>清水 愛、加藤 英美里、上坂 すみれ、戸田 めぐみ、清水 彩香、桐谷 蝶々、藤田 昌代</t>
         </is>
       </c>
       <c r="AA92" s="1" t="inlineStr">
@@ -11204,7 +11204,7 @@
       </c>
       <c r="Z100" s="1" t="inlineStr">
         <is>
-          <t>小野 涼子、清水 愛、大橋 歩夕、鹿野 まなか</t>
+          <t>北見 六花、五十鈴 みゆう、卯衣、鹿野 まなか</t>
         </is>
       </c>
       <c r="AA100" s="1" t="inlineStr">
@@ -11403,7 +11403,7 @@
           <t>水城 新人、Team-OZ、山口 朗彦、hikaru</t>
         </is>
       </c>
-      <c r="Z102" t="inlineStr">
+      <c r="Z102" s="0" t="inlineStr">
         <is>
           <t>成瀬 未亜、手塚 りょうこ</t>
         </is>
@@ -11977,7 +11977,7 @@
       </c>
       <c r="Z107" s="1" t="inlineStr">
         <is>
-          <t>浅川 悠、遥 そら、種﨑 敦美、高森 奈津美</t>
+          <t>神代 岬、遥 そら、桐谷 華、小鳥居 夕花</t>
         </is>
       </c>
       <c r="AA107" s="1" t="inlineStr">
@@ -13085,7 +13085,7 @@
       </c>
       <c r="Z117" s="1" t="inlineStr">
         <is>
-          <t>儀武 ゆう子</t>
+          <t>江口 拓也、櫻井 孝宏、村瀬 歩、儀武 ゆう子、加隈 亜衣、置鮎 龍太郎、山本 希望、原 由実、佐倉 綾音、種田 梨沙、水瀬 いのり、内田 夕夜、赤﨑 千夏、杉山 大</t>
         </is>
       </c>
       <c r="AA117" s="1" t="inlineStr">
@@ -13456,7 +13456,7 @@
       </c>
       <c r="Z120" s="1" t="inlineStr">
         <is>
-          <t>中島 沙樹、羽多野 渉、遥 そら、奏雨、高森 奈津美、猫村 ゆき</t>
+          <t>波奈束 風景、春野 風、遥 そら、奏雨、小鳥居 夕花、猫村 ゆき</t>
         </is>
       </c>
       <c r="AA120" s="1" t="inlineStr">
@@ -13902,7 +13902,7 @@
       </c>
       <c r="Z124" s="1" t="inlineStr">
         <is>
-          <t>小倉 結衣、藤森 ゆき奈、澤田 なつ、五行 なずな、大花 どん、早瀬 ゃょぃ、萌花ちょこ、藤神 司朗、猫村 ゆき、牛蛙 キタロウ</t>
+          <t>小倉 結衣、藤森 ゆき奈、澤田 なつ、五行 なずな、大花 どん、早瀬 ゃょぃ、萌花ちょこ、藤神 司朗、牛蛙 キタロウ</t>
         </is>
       </c>
       <c r="AA124" s="1" t="inlineStr">
@@ -14128,7 +14128,7 @@
       </c>
       <c r="Z126" s="1" t="inlineStr">
         <is>
-          <t>洲崎 綾</t>
+          <t>高城 みつ、佐倉 綾音、洲崎 綾</t>
         </is>
       </c>
       <c r="AA126" s="1" t="inlineStr">
@@ -14588,7 +14588,7 @@
       </c>
       <c r="Z130" s="1" t="inlineStr">
         <is>
-          <t>花澤 香菜、今井 麻美、桃井 はるこ、矢作 紗友里</t>
+          <t>田村 ゆかり、花澤 香菜、今井 麻美、宮野 真守、後藤 沙緒里、桃井 はるこ、関 智一、矢作 紗友里</t>
         </is>
       </c>
       <c r="AA130" s="1" t="inlineStr">
@@ -15153,7 +15153,7 @@
       </c>
       <c r="Z135" s="1" t="inlineStr">
         <is>
-          <t>春日 アン、柚木 サチ、新山 ゆうき</t>
+          <t>春日 アン、森谷 実園、柚木 サチ、井ノ上 花、新山 ゆうき</t>
         </is>
       </c>
       <c r="AA135" s="1" t="inlineStr">
@@ -15657,7 +15657,7 @@
       </c>
       <c r="Z140" s="1" t="inlineStr">
         <is>
-          <t>ヒマリ、中村 あむ、八木 侑紀、佐伯 伊織</t>
+          <t>ヒマリ、中村 あむ</t>
         </is>
       </c>
       <c r="AA140" s="1" t="inlineStr">
@@ -15860,7 +15860,7 @@
           <t>むにょっ、盛合 千鶴子、ポパン、秋山 裕和</t>
         </is>
       </c>
-      <c r="Z142" t="inlineStr">
+      <c r="Z142" s="0" t="inlineStr">
         <is>
           <t>真中 海、葵 時緒</t>
         </is>
@@ -16310,7 +16310,7 @@
       </c>
       <c r="Z146" s="1" t="inlineStr">
         <is>
-          <t>桐谷 華、小鳥居 夕花、鈴谷 まや、卯衣、桃山 いおん、桃園 にな、双葉 まりか</t>
+          <t>桐谷 華、小鳥居 夕花、鈴谷 まや、卯衣、桃山 いおん、桃園 にな</t>
         </is>
       </c>
       <c r="AA146" s="1" t="inlineStr">
@@ -17080,7 +17080,7 @@
       </c>
       <c r="Z153" s="1" t="inlineStr">
         <is>
-          <t>米澤 円、福圓 美里、浅倉 杏美、山本 希望</t>
+          <t>三代 眞子、澤田 なつ、紺野 由梨、瀬良 みと</t>
         </is>
       </c>
       <c r="AA153" s="1" t="inlineStr">
@@ -18153,7 +18153,7 @@
       </c>
       <c r="Z163" s="1" t="inlineStr">
         <is>
-          <t>森井 花音、野月 まひる、河村 眞人、篠原 ゆみ、井村屋 ほのか、杏 花、高橋 がならない、歩 サラ、桧鶴まき、道出 翔</t>
+          <t>柚木 かなめ、かわしま りの、原田 友貴、森井 花音、野月 まひる、河村 眞人、篠原 ゆみ、井村屋 ほのか、杏 花、高橋 がならない、歩 サラ、桧鶴まき</t>
         </is>
       </c>
       <c r="AA163" s="1" t="inlineStr">
@@ -18379,7 +18379,7 @@
       </c>
       <c r="Z165" s="1" t="inlineStr">
         <is>
-          <t>白月 かなめ、有村 祥</t>
+          <t>小倉 結衣、古河 徹人、白月 かなめ、森谷 実園、門倉 宗一、有村 祥</t>
         </is>
       </c>
       <c r="AA165" s="1" t="inlineStr">
@@ -18603,7 +18603,7 @@
           <t>Elements Garden、菊田 大介、藤間 仁、藤田 淳平、ピクセルビー、松本 文紀、母里 治樹、岩橋 星実、喜多 智弘、中山 真斗、￥Cuスタ平</t>
         </is>
       </c>
-      <c r="Z167" t="inlineStr">
+      <c r="Z167" s="0" t="inlineStr">
         <is>
           <t>雪見 そら、一色 ヒカル、民安 ともえ、楠 鈴音、羽仁 麗、岡村 美佳沙</t>
         </is>
@@ -19031,7 +19031,7 @@
           <t>Ceui、忍、菊地 創、小高 光太郎</t>
         </is>
       </c>
-      <c r="Z171" t="inlineStr">
+      <c r="Z171" s="0" t="inlineStr">
         <is>
           <t>藤森 ゆき奈、澤田 なつ、杏子 御津、加乃 みるく、外屋 舞美、美波 りお</t>
         </is>
@@ -19145,7 +19145,7 @@
       </c>
       <c r="Z172" s="1" t="inlineStr">
         <is>
-          <t>新田 恵海、宮崎 羽衣、又吉 愛、桜咲 千依、藤邑 鈴香、佐々木 未来、海保 絵果</t>
+          <t>新田 恵海、宮崎 羽衣、又吉 愛、桜咲 千依、佐々木 未来</t>
         </is>
       </c>
       <c r="AA172" s="1" t="inlineStr">
@@ -20047,7 +20047,7 @@
       </c>
       <c r="Z180" s="1" t="inlineStr">
         <is>
-          <t>石田 彰、岸尾 だいすけ、花澤 香菜、小林 ゆう、細谷 佳正、杉田 智和、安元 洋貴、福山 潤、緒方 恵美、高山 みなみ、小清水 亜美、朴 璐美、三石 琴乃、三森 すずこ、荒川 美穂、茅野 愛衣</t>
+          <t>石田 彰、岸尾 だいすけ、花澤 香菜、小林 ゆう、細谷 佳正、杉田 智和、安元 洋貴、福山 潤、\N、緒方 恵美、大山 のぶ代、高山 みなみ、小清水 亜美、朴 璐美、三石 琴乃、荒川 美穂、茅野 愛衣</t>
         </is>
       </c>
       <c r="AA180" s="1" t="inlineStr">
@@ -20386,7 +20386,7 @@
       </c>
       <c r="Z183" s="1" t="inlineStr">
         <is>
-          <t>小野 涼子、咲乃 藍里、吉田 真弓、大橋 歩夕、中村 繪里子</t>
+          <t>五行 なずな、星咲 イリア、森谷 実園、卯衣、月乃 和留都</t>
         </is>
       </c>
       <c r="AA183" s="1" t="inlineStr">
@@ -20489,7 +20489,7 @@
           <t>Elements Garden、菊田 大介、藤間 仁、藤田 淳平、母里 治樹、岩橋 星実、喜多 智弘、中山 真斗、￥Cuスタ平</t>
         </is>
       </c>
-      <c r="Z184" t="inlineStr">
+      <c r="Z184" s="0" t="inlineStr">
         <is>
           <t>雪見 そら、一色 ヒカル、民安 ともえ、かわしま りの、楠 鈴音、羽仁 麗、青山 ゆかり、岡村 美佳沙</t>
         </is>
@@ -20604,7 +20604,7 @@
       </c>
       <c r="Z185" s="1" t="inlineStr">
         <is>
-          <t>一色 ヒカル、かわしま りの、桜川 未央、野月 まひる、古河 徹人、杉原 茉莉、ますおか ゆうじ</t>
+          <t>一色 ヒカル、かわしま りの、胸肩 腎、桜川 未央、野月 まひる、古河 徹人、杉原 茉莉、ますおか ゆうじ</t>
         </is>
       </c>
       <c r="AA185" s="1" t="inlineStr">
@@ -21151,7 +21151,7 @@
       </c>
       <c r="Z190" s="1" t="inlineStr">
         <is>
-          <t>田村 ゆかり、種﨑 敦美、桃井 はるこ、岡嶋 妙、小野 涼子、清水 愛、吉田 真弓、鈴谷 まや、阿澄 佳奈</t>
+          <t>田村 ゆかり、桐谷 華、あかつき かなた、遠野 そよぎ、五行 なずな、五十鈴 みゆう、森谷 実園、鈴谷 まや、阿澄 佳奈</t>
         </is>
       </c>
       <c r="AA190" s="1" t="inlineStr">
@@ -22696,7 +22696,7 @@
       </c>
       <c r="Z204" s="0" t="inlineStr">
         <is>
-          <t>Mako</t>
+          <t>沢城 みゆき、下野 紘、柿原 徹也、今井 麻美、喜多村 英梨、中村 悠一、佐藤 利奈、杉田 智和、大谷 育江、吉田 聖子、新井 里美、Mako、山本 彩乃、南里 侑香、戸松 遥</t>
         </is>
       </c>
       <c r="AA204" s="0" t="inlineStr">
@@ -22906,7 +22906,7 @@
       </c>
       <c r="Z206" s="1" t="inlineStr">
         <is>
-          <t>青葉 りんご、桃井 いちご、いすず あすか、森谷 実園、鈴木 らん</t>
+          <t>青葉 りんご、桃井 いちご、いすず あすか、森谷 実園、鈴木 らん、日々野 蒔</t>
         </is>
       </c>
       <c r="AA206" s="1" t="inlineStr">
@@ -23570,7 +23570,7 @@
       </c>
       <c r="Z212" s="1" t="inlineStr">
         <is>
-          <t>楠 鈴音、藤森 ゆき奈、東 かりん、杏子 御津、佐本 二厘、宮沢 ゆあな、みなづき 蓮</t>
+          <t>楠 鈴音、藤森 ゆき奈、東 かりん、杏子 御津、佐本 二厘、宮沢 ゆあな</t>
         </is>
       </c>
       <c r="AA212" s="1" t="inlineStr">
@@ -23674,7 +23674,7 @@
       </c>
       <c r="Z213" s="1" t="inlineStr">
         <is>
-          <t>茶谷 やすら、遠野 そよぎ、涼森 ちさと、宮沢 ゆあな</t>
+          <t>茶谷 やすら、小倉 結衣、藤森 ゆき奈、遠野 そよぎ、涼森 ちさと、宮沢 ゆあな</t>
         </is>
       </c>
       <c r="AA213" s="1" t="inlineStr">
@@ -23878,7 +23878,7 @@
           <t>Duca、Manack</t>
         </is>
       </c>
-      <c r="Z215" t="inlineStr">
+      <c r="Z215" s="0" t="inlineStr">
         <is>
           <t>白波 遥、一色 ヒカル、姫川 あいり</t>
         </is>
@@ -24003,7 +24003,7 @@
       </c>
       <c r="Z216" s="1" t="inlineStr">
         <is>
-          <t>沢城 みゆき、小野 大輔、桑谷 夏子</t>
+          <t>沢城 みゆき、鈴村 健一、大原 さやか、小野 大輔、田村 ゆかり、大浦 冬華、小林 ゆう、釘宮 理恵、桑谷 夏子、井上 麻里奈、篠原 恵美</t>
         </is>
       </c>
       <c r="AA216" s="1" t="inlineStr">
@@ -24597,7 +24597,7 @@
           <t>Little Wing、I've、Barbarian On The Groove、SHIM、C.G Mix、尾崎 武士</t>
         </is>
       </c>
-      <c r="Z221" t="inlineStr">
+      <c r="Z221" s="0" t="inlineStr">
         <is>
           <t>さくら はづき、神村 ひな、岩田 由貴、山下 一真</t>
         </is>
@@ -24828,7 +24828,7 @@
       </c>
       <c r="Z223" s="1" t="inlineStr">
         <is>
-          <t>志村 由美、後藤 麻衣、間島 淳司、中島 裕美子、中村 繪里子、船橋 まい</t>
+          <t>志村 由美、後藤 麻衣、間島 淳司、中島 裕美子、中村 繪里子</t>
         </is>
       </c>
       <c r="AA223" s="1" t="inlineStr">
@@ -25054,7 +25054,7 @@
           <t>アッチョリケ、堀江 晶太</t>
         </is>
       </c>
-      <c r="Z225" t="inlineStr">
+      <c r="Z225" s="0" t="inlineStr">
         <is>
           <t>沢村 かすみ、たなか りお、遠野 そよぎ、五行 なずな、泉 菊之介、川椰 珱、縦溝 精史、籐野 らん、森谷 実園、みなせがわ ゆい</t>
         </is>
@@ -26029,7 +26029,7 @@
       </c>
       <c r="Z234" s="1" t="inlineStr">
         <is>
-          <t>鷹月 さくら、小手島 ひばり、有栖川 みや美、佐本 二厘、桜坂 かい、天乃 そら、水鏡</t>
+          <t>鷹月 さくら、小手島 ひばり、有栖川 みや美、佐本 二厘、桜坂 かい、天乃 そら</t>
         </is>
       </c>
       <c r="AA234" s="1" t="inlineStr">
@@ -26730,7 +26730,7 @@
       </c>
       <c r="Z240" s="1" t="inlineStr">
         <is>
-          <t>夏野 こおり、一色 ヒカル、榊原 ゆい、風音、先割れ丼、芝原 のぞみ</t>
+          <t>夏野 こおり、一色 ヒカル、榊原 ゆい、風音、先割れ丼</t>
         </is>
       </c>
       <c r="AA240" s="1" t="inlineStr">
@@ -27065,7 +27065,7 @@
       </c>
       <c r="Z243" s="1" t="inlineStr">
         <is>
-          <t>やなせ なつみ</t>
+          <t>やなせ なつみ、綾川 りの</t>
         </is>
       </c>
       <c r="AA243" s="1" t="inlineStr">
@@ -27421,7 +27421,7 @@
       </c>
       <c r="Z246" s="1" t="inlineStr">
         <is>
-          <t>田中 涼子、田宮 トモエ、緑川 光、神奈 延年、すずき けいこ、金子 明美、風音、荒井 悠美、織田 優成、柳瀬 なつみ、鴨ノ宮 ゆう</t>
+          <t>田中 涼子、田宮 トモエ、緑川 光、神奈 延年、すずき けいこ、金子 明美、風音、荒井 悠美、織田 優成、柳瀬 なつみ</t>
         </is>
       </c>
       <c r="AA246" s="1" t="inlineStr">
@@ -27639,7 +27639,7 @@
       </c>
       <c r="Z248" s="1" t="inlineStr">
         <is>
-          <t>涼宮 琉那、北都 南、草柳 順子、紫苑 みやび、佐本 二厘、石川 乃奈、篠崎 双葉、河合 春華、名塚 佳織</t>
+          <t>涼宮 琉那、北都 南、草柳 順子、紫苑 みやび、佐本 二厘、石川 乃奈、篠崎 双葉、河合 春華</t>
         </is>
       </c>
       <c r="AA248" s="1" t="inlineStr">
@@ -27872,7 +27872,7 @@
       </c>
       <c r="Z250" s="1" t="inlineStr">
         <is>
-          <t>田中 涼子、永田 佳代、たかはし 智秋、吉田 愛理、萩 道彦、相田 さやか、松園 ルイ</t>
+          <t>田中 涼子、永田 佳代、たかはし 智秋、吉田 愛理、萩 道彦、相田 さやか</t>
         </is>
       </c>
       <c r="AA250" s="1" t="inlineStr">
@@ -28517,7 +28517,7 @@
       </c>
       <c r="Z256" s="1" t="inlineStr">
         <is>
-          <t>高野 直子、氷青、生天目 仁美、後藤 麻衣、成瀬 未亜、伊藤 静、佐本 二厘、黒河 奈美</t>
+          <t>雅 姫乃、海原 エレナ、手塚 まき、安玖深 音、成瀬 未亜、三咲 里奈、佐本 二厘、本山 美奈</t>
         </is>
       </c>
       <c r="AA256" s="1" t="inlineStr">
@@ -28634,7 +28634,7 @@
       </c>
       <c r="Z257" s="1" t="inlineStr">
         <is>
-          <t>一色 ヒカル、中村 悠一、涼森 ちさと、佐々木 あかり、新田 祐一</t>
+          <t>一色 ヒカル、中村 悠一、涼森 ちさと、佐々木 あかり</t>
         </is>
       </c>
       <c r="AA257" s="1" t="inlineStr">
@@ -29287,7 +29287,7 @@
       </c>
       <c r="Z263" s="1" t="inlineStr">
         <is>
-          <t>宮崎 羽衣、中原 麻衣、深井 晴花、浅野 麻理亜、MIENO、高槻 つばさ、野川 さくら、新谷 良子、斎藤 桃子、稲村 優奈、庄子 裕衣、千葉 紗子</t>
+          <t>宮崎 羽衣、中原 麻衣、松永 雪希、深井 晴花、浅野 麻理亜、\N、\N、斎藤 桃子</t>
         </is>
       </c>
       <c r="AA263" s="1" t="inlineStr">
@@ -29939,7 +29939,7 @@
           <t>ジズスタジオ、dai、志倉 千代丸、OdiakeS、上野 浩司、磯江 俊道、5zizz、Morrigan、川越 好博、ラック眼力、zts、七瀬 光、折倉 俊則、pre-holder、SB YUNE、煉獄庭園、海老スパ、すえばし、tack、モロコ、風域、DJ NETA-RAW、朱月 笛丸、カレギュウ (oi)</t>
         </is>
       </c>
-      <c r="Z269" t="inlineStr">
+      <c r="Z269" s="0" t="inlineStr">
         <is>
           <t>小野 大輔、田村 ゆかり、保志 総一朗、中原 麻衣、雪野 五月、大川 透、関 俊彦、伊藤 美紀、かない みか</t>
         </is>
@@ -30517,7 +30517,7 @@
       </c>
       <c r="Z274" s="1" t="inlineStr">
         <is>
-          <t>紫苑 みやび</t>
+          <t>紫苑 みやび、片瀬 唯</t>
         </is>
       </c>
       <c r="AA274" s="1" t="inlineStr">
@@ -31285,7 +31285,7 @@
       </c>
       <c r="Z281" s="1" t="inlineStr">
         <is>
-          <t>笹本 優子</t>
+          <t>藤原 理加、奥田 秋、吉野 なつき、野中 真澄、北都 南、高柳 香帆、笹本 優子</t>
         </is>
       </c>
       <c r="AA281" s="1" t="inlineStr">
@@ -31386,7 +31386,7 @@
       </c>
       <c r="Z282" s="1" t="inlineStr">
         <is>
-          <t>かわしま りの、西田 こむぎ、金田 まひる、YUKI、椎名 奏子</t>
+          <t>かわしま りの、西田 こむぎ、金田 まひる、\N、椎名 奏子</t>
         </is>
       </c>
       <c r="AA282" s="1" t="inlineStr">
@@ -31999,7 +31999,7 @@
       </c>
       <c r="Z287" s="1" t="inlineStr">
         <is>
-          <t>川澄 綾子、石田 彰、まき いづみ、能登 麻美子、芹園 みや、桜木 あおい、根谷 美智子、野川 さくら、坂本 翔子、福井 裕佳梨、武下 真奈美</t>
+          <t>川澄 綾子、石田 彰、まき いづみ、能登 麻美子、根谷 美智子、福井 裕佳梨</t>
         </is>
       </c>
       <c r="AA287" s="1" t="inlineStr">
@@ -32636,7 +32636,7 @@
       </c>
       <c r="Z293" s="1" t="inlineStr">
         <is>
-          <t>比留間 京之介、北都 南、佐々 留美子、桐谷 華、桃井 穂美、七ヶ瀬 輪、平野 響子、片瀬 唯、結衣菜、杉沢 淳子、MIWAKO、桜川 美央、佐藤 涼樹</t>
+          <t>比留間 京之介、北都 南、佐々 留美子、桐谷 華、桃井 穂美、七ヶ瀬 輪、平野 響子、片瀬 唯、結衣菜、杉沢 淳子、\N、桜川 美央</t>
         </is>
       </c>
       <c r="AA293" s="1" t="inlineStr">
@@ -33076,7 +33076,7 @@
       </c>
       <c r="Z297" s="1" t="inlineStr">
         <is>
-          <t>沢城 みゆき、成田 剣、井上 喜久子、久川 綾、小清水 亜美、荻原 秀樹、こおろぎ さとみ、麻見 順子、高垣 彩陽、南 央美、岡野 浩介、入野 自由、千葉 一伸</t>
+          <t>沢城 みゆき、成田 剣、井上 喜久子、小清水 亜美、荻原 秀樹、高垣 彩陽、岡野 浩介</t>
         </is>
       </c>
       <c r="AA297" s="1" t="inlineStr">
@@ -33418,7 +33418,7 @@
       </c>
       <c r="Z300" s="1" t="inlineStr">
         <is>
-          <t>高野 直子、小林 沙苗、小田 真ゆみ</t>
+          <t>高野 直子、小林 沙苗</t>
         </is>
       </c>
       <c r="AA300" s="1" t="inlineStr">
@@ -33515,7 +33515,7 @@
       </c>
       <c r="Z301" s="1" t="inlineStr">
         <is>
-          <t>堀江 由衣、田村 ゆかり、杉田 智和、飯塚 雅弓、國府田 マリ子、小西 寛子、佐藤 朱</t>
+          <t>堀江 由衣、田村 ゆかり、杉田 智和、飯塚 雅弓、國府田 マリ子、小西 寛子</t>
         </is>
       </c>
       <c r="AA301" s="1" t="inlineStr">
@@ -33825,7 +33825,7 @@
       </c>
       <c r="Z304" s="1" t="inlineStr">
         <is>
-          <t>みる、雪野 五月、木村 あやか、芹園 みや、高森 奈津美、須本 綾奈、日下 千鶴、今井 由香、大谷 育江、飯塚 雅弓、愛美、横山 智佐、中川 亜紀子、高橋 花林、石見 舞菜香、前田 佳織里、立花 日菜</t>
+          <t>みる、雪野 五月、木村 あやか、芹園 みや、高森 奈津美、日下 千鶴、今井 由香</t>
         </is>
       </c>
       <c r="AA304" s="1" t="inlineStr">
@@ -33946,7 +33946,7 @@
       </c>
       <c r="Z305" s="1" t="inlineStr">
         <is>
-          <t>小林 ゆう、檜山 修之、井上 喜久子、釘宮 理恵、久川 綾、楠 大典、今井 由香、冬馬 由美、大塚 明夫、根谷 美智子、佐久間 レイ、内田 真礼、名塚 佳織、大西 沙織、林 勇、前田 玲奈</t>
+          <t>小林 ゆう、檜山 修之、井上 喜久子、釘宮 理恵、楠 大典、今井 由香、根谷 美智子、佐久間 レイ</t>
         </is>
       </c>
       <c r="AA305" s="1" t="inlineStr">
@@ -34059,7 +34059,7 @@
       </c>
       <c r="Z306" s="1" t="inlineStr">
         <is>
-          <t>鷹月 さくら、一宮 桜、和泉 あやか、立花 舞、今井 かおる、田中 大輔</t>
+          <t>鷹月 さくら、一宮 桜、和泉 あやか、立花 舞、今井 かおる</t>
         </is>
       </c>
       <c r="AA306" s="1" t="inlineStr">
@@ -34156,7 +34156,7 @@
       </c>
       <c r="Z307" s="1" t="inlineStr">
         <is>
-          <t>田中 敦子、北見 六花、折笠 愛、こおろぎ さとみ、秋野 花、姫川 あいり、勝生 真沙子、鶴屋 春人、鈴谷 まや、手塚 ちはる、和央 きりか、葵 時緒、山田 みほ、浅田 葉子、吉田 小南美、中村 尚子、矢島 晶子、松下 美由紀、猫村 ゆき、水沢潤、東雲 りあ、大宮 若葉、藤野 かほる、高田 由美、夏樹 柑菜、よもぎ かすみ、菊池 いづみ</t>
+          <t>田中 敦子、北見 六花、折笠 愛、こおろぎ さとみ、秋野 花、姫川 あいり、鈴谷 まや、手塚 ちはる、和央 きりか、吉田 小南美、中村 尚子、矢島 晶子、水沢潤、藤野 かほる</t>
         </is>
       </c>
       <c r="AA307" s="1" t="inlineStr">
@@ -34253,7 +34253,7 @@
       </c>
       <c r="Z308" s="1" t="inlineStr">
         <is>
-          <t>永島 由子、井上 喜久子、こおろぎ さとみ、笠原留美、高橋 美紀、平松 晶子、水谷 優子、丹下 桜、萩森 侚子、國府田 マリ子、豊嶋 真千子、渡辺菜生子、柳瀬 なつみ、深見 梨加、鈴木 真仁、小野綾子、草地 章江、小野寺麻理子</t>
+          <t>永島 由子、井上 喜久子、こおろぎ さとみ、笠原留美、高橋 美紀、平松 晶子、水谷 優子、丹下 桜、萩森 侚子、國府田 マリ子、豊嶋 真千子、渡辺菜生子、柳瀬 なつみ、深見 梨加、鈴木 真仁、小野綾子、草地 章江</t>
         </is>
       </c>
       <c r="AA308" s="1" t="inlineStr">

</xml_diff>